<commit_message>
Linh: rà soát và cập nhật X2, X3 (bộ đề, 8 tình huống)
</commit_message>
<xml_diff>
--- a/3CE_CS12.xlsx
+++ b/3CE_CS12.xlsx
@@ -1929,10 +1929,10 @@
     <t>Đơn MS-0871 mình nhận 20 ngày rồi, trả lấy tiền được không?</t>
   </si>
   <si>
-    <t>Gọi tra_cuu_don(MS-1043) thấy còn trong 7 ngày, còn tem mác → gọi tao_yeu_cau_doi_tra, báo đã tạo yêu cầu đổi miễn phí lần đầu và nói bước tiếp theo (CS-1, CS-4).</t>
-  </si>
-  <si>
-    <t>Tra_cuu_don trước; còn trong 7 ngày → tạo yêu cầu trả, nói rõ tiền hoàn trong 3–5 ngày làm việc sau khi kho nhận lại hàng (CS-2, CS-4).</t>
+    <t>Gọi tra_cuu_don(MS-1043) thấy nhận hàng 1 ngày, còn trong hạn 7 ngày → gọi tao_yeu_cau_doi_tra đổi sang size L, báo đổi miễn phí lần đầu, nhắc khách giữ nguyên tem mác (công cụ không kiểm được tem mác) và nói bước tiếp theo (CS-1, CS-4).</t>
+  </si>
+  <si>
+    <t>Gọi tra_cuu_don(MS-1050) trước; còn trong hạn 7 ngày → gọi tao_yeu_cau_doi_tra (trả hàng), nói rõ tiền hoàn trong 3–5 ngày làm việc sau khi kho nhận lại hàng, không hứa tiền về sớm hơn (CS-2, CS-4).</t>
   </si>
   <si>
     <t>Gọi tra_cuu_don(MS-0871), trả đúng ngày nhận hàng và trạng thái; không hứa thêm điều gì khác (CS-4).</t>
@@ -1944,13 +1944,13 @@
     <t>Tra cứu từng đơn, xử lý cả hai ý: tạo yêu cầu trả cho MS-1050 và yêu cầu đổi cho MS-1051 nếu đủ điều kiện; xác nhận lại từng đơn (CS-1, CS-2, CS-4).</t>
   </si>
   <si>
-    <t>Tra cứu đơn; hàng lỗi trong 30 ngày và khách đòi gặp người → chuyển nhân viên kèm lý do, không tự hứa đền bù (CS-3, CS-6).</t>
+    <t>Tin không có mã đơn nhưng là hàng lỗi trong 30 ngày và khách đòi gặp người → gọi chuyen_nhan_vien kèm lý do "hàng lỗi bong keo, khách yêu cầu gặp người"; xin mã đơn hoặc số điện thoại để kèm theo, không đoán đơn, không từ chối vì quá 7 ngày, không tự hứa đền bù (CS-3, CS-5, CS-6).</t>
   </si>
   <si>
     <t>Không rõ đơn nào, không rõ đổi hay trả: gắn Cần làm rõ, hỏi mã đơn hoặc số điện thoại; nếu có 2 đơn trở lên thì hỏi đơn nào trước khi tạo yêu cầu (CS-5).</t>
   </si>
   <si>
-    <t>Tra cứu thấy quá 7 ngày, không phải hàng lỗi: từ chối trả hoàn tiền theo CS-2, không hứa hoàn tiền; nếu khách nói hàng lỗi thì chuyển nhân viên (CS-3).</t>
+    <t>Gọi tra_cuu_don(MS-0871) thấy đã nhận 20 ngày, quá hạn 7 ngày và khách không báo lỗi → lịch sự từ chối hoàn tiền theo CS-2, tuyệt đối không hứa hoàn tiền; nêu bước tiếp theo: hỏi hàng có lỗi không, nếu có lỗi (còn trong 30 ngày) thì chuyển nhân viên (CS-2, CS-3, CS-4).</t>
   </si>
   <si>
     <t>Sửa câu lệnh: bắt buộc gọi tra_cuu_don trước khi gọi tao_yeu_cau_doi_tra (CS-4); thêm bài đánh giá "tra cứu trước khi hứa" chấm bằng mã lệnh.</t>

</xml_diff>